<commit_message>
2509 Personal Except city completed
</commit_message>
<xml_diff>
--- a/input/Profile.xlsx
+++ b/input/Profile.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Shalini\MobileAutomation\Mobile Automation _talntx\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Shalini\MobileAutomation\Talntx_MobileAutomation\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F774B6A0-31D1-4107-9385-95D5E9F0441A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9B0928-D543-41D4-B711-64F1CD563195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{27BC8E43-4EB6-4ED1-99D6-D7D447CC3B0C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{27BC8E43-4EB6-4ED1-99D6-D7D447CC3B0C}"/>
   </bookViews>
   <sheets>
     <sheet name="PersonalDetails" sheetId="1" r:id="rId1"/>
+    <sheet name="Experience" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>A+Ve</t>
   </si>
@@ -47,15 +48,9 @@
     <t>123,abc street</t>
   </si>
   <si>
-    <t>City</t>
-  </si>
-  <si>
     <t>Chennai</t>
   </si>
   <si>
-    <t>Pincode</t>
-  </si>
-  <si>
     <t>600100</t>
   </si>
   <si>
@@ -72,6 +67,18 @@
   </si>
   <si>
     <t>ProfileImage</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>pincode</t>
+  </si>
+  <si>
+    <t>Experience</t>
   </si>
 </sst>
 </file>
@@ -107,9 +114,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -444,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F873A05F-98AA-4B8C-BC99-F5F8F22A7373}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="1"/>
@@ -452,29 +460,33 @@
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
     <col min="4" max="4" width="11.5703125" customWidth="1"/>
     <col min="6" max="6" width="28.140625" customWidth="1"/>
+    <col min="7" max="7" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" t="s">
-        <v>11</v>
-      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -485,13 +497,39 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="F2" t="s">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="G2" s="2">
+        <v>36435</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5711709-A825-41DF-BBFC-C3D2136F2215}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2609 UPTO EDUCATION COMPLETION
</commit_message>
<xml_diff>
--- a/input/Profile.xlsx
+++ b/input/Profile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Shalini\MobileAutomation\Talntx_MobileAutomation\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9B0928-D543-41D4-B711-64F1CD563195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C67173A-AA22-4C89-BDC1-E53F70B35A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{27BC8E43-4EB6-4ED1-99D6-D7D447CC3B0C}"/>
   </bookViews>
@@ -37,13 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>A+Ve</t>
-  </si>
-  <si>
-    <t>Ram</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>123,abc street</t>
   </si>
@@ -57,9 +51,6 @@
     <t>"src\main\java\files\one.png"</t>
   </si>
   <si>
-    <t>BloodGroup</t>
-  </si>
-  <si>
     <t>FatherName</t>
   </si>
   <si>
@@ -79,6 +70,9 @@
   </si>
   <si>
     <t>Experience</t>
+  </si>
+  <si>
+    <t>Suriya</t>
   </si>
 </sst>
 </file>
@@ -452,60 +446,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F873A05F-98AA-4B8C-BC99-F5F8F22A7373}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-    <col min="2" max="2" width="19.7109375" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" customWidth="1"/>
-    <col min="6" max="6" width="28.140625" customWidth="1"/>
-    <col min="7" max="7" width="21.85546875" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="28.140625" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
         <v>8</v>
       </c>
       <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="E1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="2">
+      <c r="F2" s="2">
         <v>36435</v>
       </c>
     </row>
@@ -524,7 +511,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
0610 TALENTSTAUS WITHOUT TESTID
</commit_message>
<xml_diff>
--- a/input/Profile.xlsx
+++ b/input/Profile.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Shalini\MobileAutomation\Talntx_MobileAutomation\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C67173A-AA22-4C89-BDC1-E53F70B35A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA26BCEA-A391-430E-9C72-73A589B758D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{27BC8E43-4EB6-4ED1-99D6-D7D447CC3B0C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{27BC8E43-4EB6-4ED1-99D6-D7D447CC3B0C}"/>
   </bookViews>
   <sheets>
     <sheet name="PersonalDetails" sheetId="1" r:id="rId1"/>
     <sheet name="Experience" sheetId="2" r:id="rId2"/>
+    <sheet name="GovernmentID's" sheetId="3" r:id="rId3"/>
+    <sheet name="BankAccount" sheetId="4" r:id="rId4"/>
+    <sheet name="Nominee" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,55 +40,109 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>123,abc street</t>
-  </si>
-  <si>
-    <t>Chennai</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+  <si>
+    <t>"src\main\java\files\one.png"</t>
+  </si>
+  <si>
+    <t>FatherName</t>
+  </si>
+  <si>
+    <t>AddressLine</t>
+  </si>
+  <si>
+    <t>ProfileImage</t>
+  </si>
+  <si>
+    <t>DOB</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>pincode</t>
+  </si>
+  <si>
+    <t>Experience</t>
+  </si>
+  <si>
+    <t>Theni</t>
   </si>
   <si>
     <t>600100</t>
   </si>
   <si>
-    <t>"src\main\java\files\one.png"</t>
-  </si>
-  <si>
-    <t>FatherName</t>
-  </si>
-  <si>
-    <t>AddressLine</t>
-  </si>
-  <si>
-    <t>ProfileImage</t>
-  </si>
-  <si>
-    <t>DOB</t>
-  </si>
-  <si>
-    <t>city</t>
-  </si>
-  <si>
-    <t>pincode</t>
-  </si>
-  <si>
-    <t>Experience</t>
-  </si>
-  <si>
-    <t>Suriya</t>
+    <t>123,ABCC street</t>
+  </si>
+  <si>
+    <t>Rakesh</t>
+  </si>
+  <si>
+    <t>Aadhar Number</t>
+  </si>
+  <si>
+    <t>PAN Number</t>
+  </si>
+  <si>
+    <t>664100722828</t>
+  </si>
+  <si>
+    <t>MNEPS5055C</t>
+  </si>
+  <si>
+    <t>Bank Name</t>
+  </si>
+  <si>
+    <t>Account Holder Name</t>
+  </si>
+  <si>
+    <t>Siran</t>
+  </si>
+  <si>
+    <t>Branch Name</t>
+  </si>
+  <si>
+    <t>Adyar</t>
+  </si>
+  <si>
+    <t>IFSC</t>
+  </si>
+  <si>
+    <t>HDFC000128</t>
+  </si>
+  <si>
+    <t>HDFC Bank</t>
+  </si>
+  <si>
+    <t>Nominee Name</t>
+  </si>
+  <si>
+    <t>Swetha</t>
+  </si>
+  <si>
+    <t>Nominee Aadhar Number</t>
+  </si>
+  <si>
+    <t>234567890989</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF5C92FF"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -108,10 +165,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,7 +507,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F873A05F-98AA-4B8C-BC99-F5F8F22A7373}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" customWidth="1"/>
@@ -456,41 +516,41 @@
     <col min="6" max="6" width="21.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>11</v>
       </c>
       <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
         <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>3</v>
       </c>
       <c r="F2" s="2">
         <v>36435</v>
@@ -504,19 +564,123 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5711709-A825-41DF-BBFC-C3D2136F2215}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
       <c r="A2">
-        <v>2</v>
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{251DA4A6-0702-425D-BA46-D964AFC40BBB}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F81F9FC1-2703-4DE8-A719-4A5AB8CEB82F}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BB4C1B9-DE5B-4980-8463-882AC6CEAB80}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="33.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
0910 TALENTSTAUS AND SIGNUP
</commit_message>
<xml_diff>
--- a/input/Profile.xlsx
+++ b/input/Profile.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Shalini\MobileAutomation\Talntx_MobileAutomation\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA26BCEA-A391-430E-9C72-73A589B758D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F72E49E-7E29-4D23-B2E0-307C1D8151D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{27BC8E43-4EB6-4ED1-99D6-D7D447CC3B0C}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>"src\main\java\files\one.png"</t>
   </si>
@@ -75,9 +75,6 @@
     <t>123,ABCC street</t>
   </si>
   <si>
-    <t>Rakesh</t>
-  </si>
-  <si>
     <t>Aadhar Number</t>
   </si>
   <si>
@@ -108,22 +105,34 @@
     <t>IFSC</t>
   </si>
   <si>
-    <t>HDFC000128</t>
-  </si>
-  <si>
     <t>HDFC Bank</t>
   </si>
   <si>
     <t>Nominee Name</t>
   </si>
   <si>
-    <t>Swetha</t>
-  </si>
-  <si>
     <t>Nominee Aadhar Number</t>
   </si>
   <si>
     <t>234567890989</t>
+  </si>
+  <si>
+    <t>HDFC0000128</t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>Suraj</t>
+  </si>
+  <si>
+    <t>123/F2 ABC Street</t>
+  </si>
+  <si>
+    <t>Chennai</t>
+  </si>
+  <si>
+    <t>Address</t>
   </si>
 </sst>
 </file>
@@ -538,7 +547,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -595,18 +604,18 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
         <v>12</v>
-      </c>
-      <c r="B1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
         <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -627,30 +636,30 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -660,27 +669,46 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BB4C1B9-DE5B-4980-8463-882AC6CEAB80}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="33.85546875" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>27</v>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2">
+        <v>600100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>